<commit_message>
Add API test scripts and remove tracked Xcode user state
- Add test scripts for Suno, Replicate, and full pipeline testing
- Add test audio file for preview testing
- Remove xcuserstate from tracking (now properly gitignored)
- Update references document

Co-authored by Ambrose Obimma
</commit_message>
<xml_diff>
--- a/references.xlsx
+++ b/references.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ao/Documents/projects/porizo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B90213B3-9136-D94A-AB32-6B5528F8CF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB988A53-77FE-464A-8E59-E2743A2B519B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4060" yWindow="3260" windowWidth="27240" windowHeight="16180" activeTab="1" xr2:uid="{E788F47F-FDDE-384F-B0C9-77A46848F202}"/>
+    <workbookView xWindow="4060" yWindow="3260" windowWidth="27240" windowHeight="16180" xr2:uid="{E788F47F-FDDE-384F-B0C9-77A46848F202}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>https://www.soundverse.ai/?tool=ai-song-generator</t>
   </si>
@@ -73,6 +73,33 @@
   </si>
   <si>
     <t>sk_f6557aa744657cc9943ced3948a231b6124f69b4307ffff4</t>
+  </si>
+  <si>
+    <t>Elevanlabs</t>
+  </si>
+  <si>
+    <t>Replicate</t>
+  </si>
+  <si>
+    <t>r8_ZSoMEf63CRJo18kif4MqecvHCsHJmab1ASyDa</t>
+  </si>
+  <si>
+    <t>Sources:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - https://cartesia.ai/learn/top-elevenlabs-alternatives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - https://suno.com/pricing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - https://www.musicful.ai/vs/suno-vs-udio/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - https://www.resemble.ai/alternative-to-elevenlabs/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - https://www.mureka.ai/hub/aimusic/best-ai-music-generator/</t>
   </si>
 </sst>
 </file>
@@ -455,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CED0EAA-974E-A544-A087-7810A75606C6}">
-  <dimension ref="C11:D19"/>
+  <dimension ref="C11:D28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="11" spans="3:4" x14ac:dyDescent="0.2">
@@ -502,6 +529,36 @@
     <row r="19" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D19" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D26" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D28" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -516,9 +573,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A043CFB-AE2B-9643-8D32-3945B3F84B29}">
-  <dimension ref="C9:D10"/>
+  <dimension ref="C7:D18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C9" t="s">
         <v>10</v>
@@ -530,6 +592,16 @@
     <row r="10" spans="3:4" x14ac:dyDescent="0.2">
       <c r="D10" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D18" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>